<commit_message>
docs(fase2): alinea entregables con Retro S03 cerrada y RNF 1.0.2
Sincroniza Word/md 2.3-2.6 e individuales con acta S03 (15/10), Goal Parcial y catálogo v1.0.2; DOC-07 Pruebas S03 v0.4; reemplaza § por ver Seccion y em dash por guion; añade scripts fase2/_tools. Actas S01/S02 firmadas sin reescribir.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/fase2/Evidencias Proyecto/Evidencias de Documentacion/03_Sprint_Backlog/Sprint_01/DPAY3_Sprint_Backlog_S01.xlsx
+++ b/fase2/Evidencias Proyecto/Evidencias de Documentacion/03_Sprint_Backlog/Sprint_01/DPAY3_Sprint_Backlog_S01.xlsx
@@ -530,7 +530,7 @@
     <row r="2" ht="48" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Sprint Backlog — D-PAY 3.0 — Sprint 1 (Semanas 5 y 6, 08/09/2026 – 21/09/2026)</t>
+          <t>Sprint Backlog - D-PAY 3.0 - Sprint 1 (Semanas 5 y 6, 08/09/2026 – 21/09/2026)</t>
         </is>
       </c>
       <c r="E2" s="3" t="inlineStr">
@@ -539,6 +539,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4" ht="22" customHeight="1">
       <c r="A4" s="4" t="inlineStr">
         <is>
@@ -607,7 +608,7 @@
       </c>
       <c r="F5" s="5" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>-</t>
         </is>
       </c>
       <c r="G5" s="5" t="inlineStr">
@@ -1312,6 +1313,7 @@
         <v/>
       </c>
     </row>
+    <row r="24"/>
     <row r="25" ht="48" customHeight="1">
       <c r="A25" s="11" t="inlineStr">
         <is>

</xml_diff>